<commit_message>
Apply Jeuz's updated workbooks and profile corrections
Replace the four models with his updated files (same values; the
Precedents and DCF workbooks drop their supporting company sheets).
Update the headline and About text, show enterprise value ranges for
the comps, precedents, and DCF results, and ignore the docs/updated/
staging folder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Merger Consequences Analysis.xlsx
+++ b/docs/Merger Consequences Analysis.xlsx
@@ -1055,7 +1055,6 @@
       <sz val="20.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font/>
     <font>
@@ -1063,81 +1062,68 @@
       <sz val="14.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <sz val="9.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1257,82 +1243,61 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="123">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="6" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="4" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="164" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="164" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="166" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0"/>
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="167" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="167" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="168" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="168" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="6" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="6" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="3" fontId="6" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="167" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="167" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="4" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="3" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="5" fillId="3" fontId="7" numFmtId="167" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="7" fillId="3" fontId="6" numFmtId="167" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
@@ -1340,37 +1305,26 @@
     <xf borderId="5" fillId="3" fontId="7" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="7" numFmtId="167" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="169" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="4" fillId="3" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="3" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="7" numFmtId="168" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="7" numFmtId="168" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="3" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="4" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="5" fontId="7" numFmtId="168" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="5" fontId="7" numFmtId="170" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="7" numFmtId="166" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="6" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="6" fillId="4" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="5" fontId="7" numFmtId="10" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="5" fontId="7" numFmtId="171" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1380,196 +1334,128 @@
     <xf borderId="8" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="6" fillId="3" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="3" fontId="10" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="10" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="4" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="3" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="2" fillId="3" fontId="6" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="9" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="10" fillId="3" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="171" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="3" fillId="3" fontId="6" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="171" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="3" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="4" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="11" fillId="3" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="7" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="7" fillId="3" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="7" fillId="3" fontId="6" numFmtId="171" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="171" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="3" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="7" numFmtId="164" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="3" fontId="6" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="15" numFmtId="167" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="3" fontId="15" numFmtId="167" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="2" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="5" fillId="3" fontId="6" numFmtId="2" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="9" fillId="3" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="7" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="7" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="7" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="4" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="13" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="3" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="3" fontId="6" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="3" fontId="13" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="13" numFmtId="164" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="3" fontId="13" numFmtId="166" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="5" fillId="3" fontId="13" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="7" fillId="3" fontId="6" numFmtId="2" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="8" fillId="3" fontId="6" numFmtId="2" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="4" fillId="3" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="15" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="5" fillId="3" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="6" fillId="3" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="3" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="7" fillId="3" fontId="10" numFmtId="166" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="10" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="166" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="166" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="6" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="6" fillId="3" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="8" fillId="3" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="6" fillId="3" fontId="13" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="8" fillId="3" fontId="13" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="3" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="6" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="3" fontId="13" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="3" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="3" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="165" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="7" fillId="3" fontId="6" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="8" fillId="3" fontId="6" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="7" fillId="3" fontId="7" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="7" fillId="3" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
@@ -1788,7 +1674,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="24.5"/>
     <col customWidth="1" min="2" max="2" width="24.88"/>
@@ -1807,7 +1693,7 @@
     <col customWidth="1" min="20" max="23" width="12.63"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1834,13 +1720,13 @@
       <c r="V1" s="2"/>
       <c r="W1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="W2" s="5"/>
     </row>
-    <row r="3">
+    <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -1867,7 +1753,8 @@
       <c r="V3" s="7"/>
       <c r="W3" s="8"/>
     </row>
-    <row r="5">
+    <row r="4" ht="15.75" customHeight="1"/>
+    <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
@@ -1898,7 +1785,7 @@
       <c r="V5" s="2"/>
       <c r="W5" s="3"/>
     </row>
-    <row r="6">
+    <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="12"/>
       <c r="B6" s="13" t="s">
         <v>8</v>
@@ -1909,10 +1796,10 @@
       <c r="D6" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="15">
         <f>B7</f>
         <v>2.28</v>
       </c>
@@ -1920,7 +1807,7 @@
       <c r="J6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="16" t="s">
         <v>13</v>
       </c>
       <c r="M6" s="12"/>
@@ -1933,7 +1820,7 @@
       <c r="P6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="Q6" s="17" t="s">
+      <c r="Q6" s="16" t="s">
         <v>17</v>
       </c>
       <c r="S6" s="12"/>
@@ -1943,241 +1830,241 @@
       <c r="V6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="W6" s="17" t="s">
+      <c r="W6" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="s">
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="17">
         <v>2.28</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="17">
         <v>0.7</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="12"/>
-      <c r="G7" s="20"/>
-      <c r="I7" s="15" t="s">
+      <c r="G7" s="19"/>
+      <c r="I7" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J7" s="21">
+      <c r="J7" s="17">
         <f>D43</f>
         <v>19585.79</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="20">
         <f t="shared" ref="K7:K10" si="3">J7/$J$11</f>
         <v>0.9828009828</v>
       </c>
-      <c r="M7" s="15" t="s">
+      <c r="M7" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="N7" s="21">
+      <c r="N7" s="17">
         <f t="shared" ref="N7:O7" si="1">B13</f>
         <v>22756.22</v>
       </c>
-      <c r="O7" s="21">
+      <c r="O7" s="17">
         <f t="shared" si="1"/>
         <v>7490.27</v>
       </c>
-      <c r="P7" s="23">
+      <c r="P7" s="21">
         <f>-J15</f>
         <v>-2301.330325</v>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="15">
         <f t="shared" ref="Q7:Q14" si="4">SUM(N7:P7)</f>
         <v>27945.15968</v>
       </c>
-      <c r="S7" s="15" t="s">
+      <c r="S7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="U7" s="24">
+      <c r="U7" s="22">
         <f t="shared" ref="U7:W7" si="2">$B$8</f>
         <v>32429.88</v>
       </c>
-      <c r="V7" s="24">
+      <c r="V7" s="22">
         <f t="shared" si="2"/>
         <v>32429.88</v>
       </c>
-      <c r="W7" s="25">
+      <c r="W7" s="23">
         <f t="shared" si="2"/>
         <v>32429.88</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="15" t="s">
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="26">
+      <c r="B8" s="24">
         <v>32429.88</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="24">
         <v>22383.76</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="25">
         <f>D53/G6</f>
         <v>5583.668202</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="26">
+      <c r="J8" s="24">
         <v>0.0</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M8" s="15" t="s">
+      <c r="M8" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="N8" s="26">
+      <c r="N8" s="24">
         <v>86530.22</v>
       </c>
-      <c r="O8" s="26">
+      <c r="O8" s="24">
         <v>4912.95</v>
       </c>
-      <c r="P8" s="26">
+      <c r="P8" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="25">
         <f t="shared" si="4"/>
         <v>91443.17</v>
       </c>
-      <c r="S8" s="15" t="s">
+      <c r="S8" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="U8" s="28">
+      <c r="U8" s="26">
         <f t="shared" ref="U8:W8" si="5">B30</f>
         <v>0.6685</v>
       </c>
-      <c r="V8" s="28">
+      <c r="V8" s="26">
         <f t="shared" si="5"/>
         <v>0.7012</v>
       </c>
-      <c r="W8" s="29">
+      <c r="W8" s="27">
         <f t="shared" si="5"/>
         <v>0.7174</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="30" t="s">
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="31">
+      <c r="B9" s="29">
         <f t="shared" ref="B9:C9" si="6">B7*B8</f>
         <v>73940.1264</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="29">
         <f t="shared" si="6"/>
         <v>15668.632</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="30" t="s">
+      <c r="F9" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="33">
+      <c r="G9" s="31">
         <f>B8</f>
         <v>32429.88</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J9" s="34">
+      <c r="J9" s="24">
         <f>D54*G24</f>
         <v>293.78685</v>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="20">
         <f t="shared" si="3"/>
         <v>0.01474201474</v>
       </c>
-      <c r="M9" s="15" t="s">
+      <c r="M9" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="N9" s="26">
+      <c r="N9" s="24">
         <v>34981.68</v>
       </c>
-      <c r="O9" s="26">
+      <c r="O9" s="24">
         <v>11679.93</v>
       </c>
-      <c r="P9" s="26">
+      <c r="P9" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="25">
         <f t="shared" si="4"/>
         <v>46661.61</v>
       </c>
       <c r="S9" s="12"/>
-      <c r="U9" s="35"/>
-      <c r="V9" s="35"/>
-      <c r="W9" s="20"/>
-    </row>
-    <row r="10">
-      <c r="F10" s="36" t="s">
+      <c r="U9" s="32"/>
+      <c r="V9" s="32"/>
+      <c r="W9" s="19"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="F10" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="34">
         <f>G8+G9</f>
         <v>38013.5482</v>
       </c>
-      <c r="I10" s="30" t="s">
+      <c r="I10" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="J10" s="38">
+      <c r="J10" s="35">
         <f>D52*G25</f>
         <v>48.964475</v>
       </c>
-      <c r="K10" s="39">
+      <c r="K10" s="36">
         <f t="shared" si="3"/>
         <v>0.002457002457</v>
       </c>
-      <c r="M10" s="15" t="s">
+      <c r="M10" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="N10" s="26">
+      <c r="N10" s="24">
         <v>139412.4</v>
       </c>
-      <c r="O10" s="26">
+      <c r="O10" s="24">
         <v>75078.68</v>
       </c>
-      <c r="P10" s="34">
+      <c r="P10" s="24">
         <f t="shared" ref="P10:P11" si="9">J26</f>
         <v>5000</v>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="25">
         <f t="shared" si="4"/>
         <v>219491.08</v>
       </c>
-      <c r="S10" s="30" t="s">
+      <c r="S10" s="28" t="s">
         <v>39</v>
       </c>
       <c r="T10" s="7"/>
-      <c r="U10" s="38">
+      <c r="U10" s="35">
         <f t="shared" ref="U10:W10" si="7">$G$8</f>
         <v>5583.668202</v>
       </c>
-      <c r="V10" s="38">
+      <c r="V10" s="35">
         <f t="shared" si="7"/>
         <v>5583.668202</v>
       </c>
-      <c r="W10" s="33">
+      <c r="W10" s="31">
         <f t="shared" si="7"/>
         <v>5583.668202</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="9" t="s">
         <v>40</v>
       </c>
@@ -2185,52 +2072,52 @@
       <c r="C11" s="2"/>
       <c r="D11" s="3"/>
       <c r="F11" s="12"/>
-      <c r="G11" s="20"/>
-      <c r="I11" s="36" t="s">
+      <c r="G11" s="19"/>
+      <c r="I11" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="40">
+      <c r="J11" s="37">
         <f t="shared" ref="J11:K11" si="8">SUM(J7:J10)</f>
         <v>19928.54133</v>
       </c>
-      <c r="K11" s="41">
+      <c r="K11" s="38">
         <f t="shared" si="8"/>
         <v>1</v>
       </c>
-      <c r="M11" s="15" t="s">
+      <c r="M11" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="N11" s="26">
+      <c r="N11" s="24">
         <v>155706.67</v>
       </c>
-      <c r="O11" s="26">
+      <c r="O11" s="24">
         <v>88813.46</v>
       </c>
-      <c r="P11" s="34">
+      <c r="P11" s="24">
         <f t="shared" si="9"/>
         <v>10000</v>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="25">
         <f t="shared" si="4"/>
         <v>254520.13</v>
       </c>
-      <c r="S11" s="36" t="s">
+      <c r="S11" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="U11" s="42">
+      <c r="U11" s="39">
         <f t="shared" ref="U11:W11" si="10">U7+U10</f>
         <v>38013.5482</v>
       </c>
-      <c r="V11" s="42">
+      <c r="V11" s="39">
         <f t="shared" si="10"/>
         <v>38013.5482</v>
       </c>
-      <c r="W11" s="37">
+      <c r="W11" s="34">
         <f t="shared" si="10"/>
         <v>38013.5482</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="12"/>
       <c r="B12" s="13" t="s">
         <v>44</v>
@@ -2241,285 +2128,285 @@
       <c r="D12" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="20">
         <f>G8/G10</f>
         <v>0.1468862673</v>
       </c>
       <c r="I12" s="12"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="20"/>
-      <c r="M12" s="15" t="s">
+      <c r="J12" s="32"/>
+      <c r="K12" s="19"/>
+      <c r="M12" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="N12" s="26">
+      <c r="N12" s="24">
         <v>12652.61</v>
       </c>
-      <c r="O12" s="26">
+      <c r="O12" s="24">
         <v>5815.92</v>
       </c>
-      <c r="P12" s="26">
+      <c r="P12" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q12" s="27">
+      <c r="Q12" s="25">
         <f t="shared" si="4"/>
         <v>18468.53</v>
       </c>
       <c r="S12" s="12"/>
-      <c r="U12" s="35"/>
-      <c r="V12" s="35"/>
-      <c r="W12" s="20"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="s">
+      <c r="U12" s="32"/>
+      <c r="V12" s="32"/>
+      <c r="W12" s="19"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="18">
+      <c r="B13" s="17">
         <v>22756.22</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="17">
         <v>7490.27</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="44">
+      <c r="G13" s="41">
         <f>G8/C8</f>
         <v>0.2494517544</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="17">
         <f t="shared" ref="J13:J14" si="12">D52</f>
         <v>4896.4475</v>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="20">
         <f t="shared" ref="K13:K15" si="13">J13/$J$16</f>
         <v>0.2457002457</v>
       </c>
-      <c r="M13" s="15" t="s">
+      <c r="M13" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="N13" s="26">
+      <c r="N13" s="24">
         <v>0.0</v>
       </c>
-      <c r="O13" s="34">
+      <c r="O13" s="24">
         <f>J38</f>
         <v>4567.24</v>
       </c>
-      <c r="P13" s="34">
+      <c r="P13" s="24">
         <f>-J38</f>
         <v>-4567.24</v>
       </c>
-      <c r="Q13" s="27">
+      <c r="Q13" s="25">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S13" s="45" t="s">
+      <c r="S13" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="U13" s="46">
+      <c r="U13" s="43">
         <f t="shared" ref="U13:W13" si="11">N56/U11</f>
         <v>0.6806875183</v>
       </c>
-      <c r="V13" s="46">
+      <c r="V13" s="43">
         <f t="shared" si="11"/>
         <v>0.7127221496</v>
       </c>
-      <c r="W13" s="47">
+      <c r="W13" s="44">
         <f t="shared" si="11"/>
         <v>0.7119822818</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="12"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="48"/>
-      <c r="F14" s="49" t="s">
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="45"/>
+      <c r="F14" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="34">
+      <c r="J14" s="24">
         <f t="shared" si="12"/>
         <v>12730.7635</v>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="20">
         <f t="shared" si="13"/>
         <v>0.6388206388</v>
       </c>
-      <c r="M14" s="30" t="s">
+      <c r="M14" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="N14" s="50">
+      <c r="N14" s="35">
         <v>50426.42</v>
       </c>
-      <c r="O14" s="50">
+      <c r="O14" s="35">
         <v>20681.83</v>
       </c>
-      <c r="P14" s="50">
+      <c r="P14" s="35">
         <v>0.0</v>
       </c>
-      <c r="Q14" s="33">
+      <c r="Q14" s="31">
         <f t="shared" si="4"/>
         <v>71108.25</v>
       </c>
-      <c r="S14" s="51" t="s">
+      <c r="S14" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="U14" s="52">
+      <c r="U14" s="48">
         <f t="shared" ref="U14:W14" si="14">U13-U8</f>
         <v>0.01218751829</v>
       </c>
-      <c r="V14" s="52">
+      <c r="V14" s="48">
         <f t="shared" si="14"/>
         <v>0.01152214956</v>
       </c>
-      <c r="W14" s="53">
+      <c r="W14" s="49">
         <f t="shared" si="14"/>
         <v>-0.00541771823</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="15" t="s">
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="26">
+      <c r="B15" s="24">
         <v>21006.56</v>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="24">
         <v>25027.21</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="49" t="s">
+      <c r="F15" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="I15" s="30" t="s">
+      <c r="I15" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="J15" s="38">
+      <c r="J15" s="35">
         <f>D51+J9+J10</f>
         <v>2301.330325</v>
       </c>
-      <c r="K15" s="39">
+      <c r="K15" s="36">
         <f t="shared" si="13"/>
         <v>0.1154791155</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="N15" s="40">
+      <c r="N15" s="37">
         <f t="shared" ref="N15:Q15" si="15">SUM(N7:N14)</f>
         <v>502466.22</v>
       </c>
-      <c r="O15" s="40">
+      <c r="O15" s="37">
         <f t="shared" si="15"/>
         <v>219040.28</v>
       </c>
-      <c r="P15" s="54">
+      <c r="P15" s="50">
         <f t="shared" si="15"/>
         <v>8131.429675</v>
       </c>
-      <c r="Q15" s="55">
+      <c r="Q15" s="51">
         <f t="shared" si="15"/>
         <v>729637.9297</v>
       </c>
-      <c r="S15" s="56" t="s">
+      <c r="S15" s="52" t="s">
         <v>62</v>
       </c>
       <c r="T15" s="7"/>
-      <c r="U15" s="57">
+      <c r="U15" s="53">
         <f t="shared" ref="U15:W15" si="16">U14/U8</f>
         <v>0.0182311418</v>
       </c>
-      <c r="V15" s="57">
+      <c r="V15" s="53">
         <f t="shared" si="16"/>
         <v>0.01643204444</v>
       </c>
-      <c r="W15" s="58">
+      <c r="W15" s="54">
         <f t="shared" si="16"/>
         <v>-0.007551879328</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="30" t="s">
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="50">
+      <c r="B16" s="35">
         <v>77873.07</v>
       </c>
-      <c r="C16" s="50">
+      <c r="C16" s="35">
         <v>61853.07</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="D16" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="I16" s="36" t="s">
+      <c r="I16" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="J16" s="40">
+      <c r="J16" s="37">
         <f t="shared" ref="J16:K16" si="17">SUM(J13:J15)</f>
         <v>19928.54133</v>
       </c>
-      <c r="K16" s="41">
+      <c r="K16" s="38">
         <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="M16" s="12"/>
-      <c r="N16" s="35"/>
-      <c r="O16" s="35"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="60"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="s">
+      <c r="N16" s="32"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="32"/>
+      <c r="Q16" s="56"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="17">
         <f t="shared" ref="B17:C17" si="18">SUM(B15:B16)</f>
         <v>98879.63</v>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="17">
         <f t="shared" si="18"/>
         <v>86880.28</v>
       </c>
-      <c r="D17" s="61"/>
+      <c r="D17" s="57"/>
       <c r="F17" s="10" t="s">
         <v>67</v>
       </c>
       <c r="G17" s="3"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="20"/>
-      <c r="M17" s="15" t="s">
+      <c r="J17" s="32"/>
+      <c r="K17" s="19"/>
+      <c r="M17" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="N17" s="18">
+      <c r="N17" s="17">
         <f t="shared" ref="N17:O17" si="19">B15</f>
         <v>21006.56</v>
       </c>
-      <c r="O17" s="18">
+      <c r="O17" s="17">
         <f t="shared" si="19"/>
         <v>25027.21</v>
       </c>
-      <c r="P17" s="18">
+      <c r="P17" s="17">
         <v>0.0</v>
       </c>
-      <c r="Q17" s="16">
+      <c r="Q17" s="15">
         <f t="shared" ref="Q17:Q24" si="21">SUM(N17:P17)</f>
         <v>46033.77</v>
       </c>
-      <c r="R17" s="62"/>
+      <c r="R17" s="58"/>
       <c r="S17" s="11" t="s">
         <v>69</v>
       </c>
@@ -2529,45 +2416,45 @@
       <c r="W17" s="2"/>
       <c r="X17" s="3"/>
     </row>
-    <row r="18">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="12"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="63"/>
-      <c r="F18" s="15" t="s">
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="59"/>
+      <c r="F18" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="64">
+      <c r="G18" s="20">
         <v>0.0675</v>
       </c>
-      <c r="I18" s="65" t="s">
+      <c r="I18" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="J18" s="66">
+      <c r="J18" s="61">
         <f t="shared" ref="J18:K18" si="20">J11-J16</f>
         <v>0</v>
       </c>
-      <c r="K18" s="67">
+      <c r="K18" s="62">
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="M18" s="15" t="s">
+      <c r="M18" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="N18" s="26">
+      <c r="N18" s="24">
         <v>34233.28</v>
       </c>
-      <c r="O18" s="26">
+      <c r="O18" s="24">
         <v>11312.58</v>
       </c>
-      <c r="P18" s="26">
+      <c r="P18" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q18" s="27">
+      <c r="Q18" s="25">
         <f t="shared" si="21"/>
         <v>45545.86</v>
       </c>
-      <c r="S18" s="68"/>
+      <c r="S18" s="63"/>
       <c r="T18" s="13" t="s">
         <v>73</v>
       </c>
@@ -2576,321 +2463,321 @@
       <c r="W18" s="7"/>
       <c r="X18" s="8"/>
     </row>
-    <row r="19">
-      <c r="A19" s="69" t="s">
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="64" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="70">
+      <c r="B19" s="65">
         <f t="shared" ref="B19:C19" si="22">B17-B13</f>
         <v>76123.41</v>
       </c>
-      <c r="C19" s="70">
+      <c r="C19" s="65">
         <f t="shared" si="22"/>
         <v>79390.01</v>
       </c>
-      <c r="D19" s="43"/>
-      <c r="F19" s="15" t="s">
+      <c r="D19" s="40"/>
+      <c r="F19" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G19" s="64">
+      <c r="G19" s="20">
         <v>0.05</v>
       </c>
-      <c r="I19" s="71" t="s">
+      <c r="I19" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="M19" s="15" t="s">
+      <c r="M19" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="N19" s="26">
+      <c r="N19" s="24">
         <v>19268.95</v>
       </c>
-      <c r="O19" s="26">
+      <c r="O19" s="24">
         <v>790.73</v>
       </c>
-      <c r="P19" s="26">
+      <c r="P19" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q19" s="27">
+      <c r="Q19" s="25">
         <f t="shared" si="21"/>
         <v>20059.68</v>
       </c>
-      <c r="S19" s="72" t="s">
+      <c r="S19" s="66" t="s">
         <v>78</v>
       </c>
-      <c r="T19" s="73">
+      <c r="T19" s="67">
         <v>0.35</v>
       </c>
-      <c r="U19" s="73">
+      <c r="U19" s="67">
         <v>0.5</v>
       </c>
-      <c r="V19" s="74">
+      <c r="V19" s="68">
         <v>0.65</v>
       </c>
-      <c r="W19" s="73">
+      <c r="W19" s="67">
         <v>0.8</v>
       </c>
-      <c r="X19" s="75">
+      <c r="X19" s="69">
         <v>1.0</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="12"/>
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="61"/>
-      <c r="F20" s="15" t="s">
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="57"/>
+      <c r="F20" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="G20" s="64">
+      <c r="G20" s="20">
         <v>0.25</v>
       </c>
-      <c r="I20" s="71" t="s">
+      <c r="I20" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="M20" s="15" t="s">
+      <c r="M20" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="N20" s="26">
+      <c r="N20" s="24">
         <f t="shared" ref="N20:O20" si="23">B16</f>
         <v>77873.07</v>
       </c>
-      <c r="O20" s="26">
+      <c r="O20" s="24">
         <f t="shared" si="23"/>
         <v>61853.07</v>
       </c>
-      <c r="P20" s="26">
+      <c r="P20" s="24">
         <f>J13-J10</f>
         <v>4847.483025</v>
       </c>
-      <c r="Q20" s="27">
+      <c r="Q20" s="25">
         <f t="shared" si="21"/>
         <v>144573.623</v>
       </c>
-      <c r="S20" s="76">
+      <c r="S20" s="70">
         <v>0.15</v>
       </c>
-      <c r="T20" s="77">
+      <c r="T20" s="71">
         <v>0.0888</v>
       </c>
-      <c r="U20" s="77">
+      <c r="U20" s="71">
         <v>0.0592</v>
       </c>
-      <c r="V20" s="78">
+      <c r="V20" s="72">
         <v>0.0314</v>
       </c>
-      <c r="W20" s="77">
+      <c r="W20" s="71">
         <v>0.0054</v>
       </c>
-      <c r="X20" s="79">
+      <c r="X20" s="73">
         <v>-0.028</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="s">
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="17">
         <v>320667.32</v>
       </c>
-      <c r="C21" s="18">
+      <c r="C21" s="17">
         <v>97123.48</v>
       </c>
-      <c r="D21" s="61"/>
-      <c r="F21" s="69" t="s">
+      <c r="D21" s="57"/>
+      <c r="F21" s="64" t="s">
         <v>83</v>
       </c>
-      <c r="G21" s="80">
+      <c r="G21" s="74">
         <f>G18*(1-G20)</f>
         <v>0.050625</v>
       </c>
-      <c r="I21" s="71" t="s">
+      <c r="I21" s="58" t="s">
         <v>84</v>
       </c>
-      <c r="M21" s="15" t="s">
+      <c r="M21" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="N21" s="26">
+      <c r="N21" s="24">
         <v>17942.99</v>
       </c>
-      <c r="O21" s="26">
+      <c r="O21" s="24">
         <v>4191.65</v>
       </c>
-      <c r="P21" s="26">
+      <c r="P21" s="24">
         <f>J30</f>
         <v>3750</v>
       </c>
-      <c r="Q21" s="27">
+      <c r="Q21" s="25">
         <f t="shared" si="21"/>
         <v>25884.64</v>
       </c>
-      <c r="S21" s="76">
+      <c r="S21" s="70">
         <v>0.2</v>
       </c>
-      <c r="T21" s="77">
+      <c r="T21" s="71">
         <v>0.084</v>
       </c>
-      <c r="U21" s="77">
+      <c r="U21" s="71">
         <v>0.0534</v>
       </c>
-      <c r="V21" s="78">
+      <c r="V21" s="72">
         <v>0.0248</v>
       </c>
-      <c r="W21" s="81">
+      <c r="W21" s="75">
         <v>-0.002</v>
       </c>
-      <c r="X21" s="79">
+      <c r="X21" s="73">
         <v>-0.0363</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="30" t="s">
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="B22" s="82">
+      <c r="B22" s="29">
         <v>284350.55</v>
       </c>
-      <c r="C22" s="82">
+      <c r="C22" s="29">
         <v>92618.9</v>
       </c>
-      <c r="D22" s="59" t="s">
+      <c r="D22" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="20">
         <f>G19*(1-G20)</f>
         <v>0.0375</v>
       </c>
-      <c r="I22" s="71" t="s">
+      <c r="I22" s="58" t="s">
         <v>89</v>
       </c>
-      <c r="M22" s="83" t="s">
+      <c r="M22" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="N22" s="26">
+      <c r="N22" s="24">
         <v>0.0</v>
       </c>
-      <c r="O22" s="26">
+      <c r="O22" s="24">
         <v>11420.08</v>
       </c>
-      <c r="P22" s="26">
+      <c r="P22" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q22" s="27">
+      <c r="Q22" s="25">
         <f t="shared" si="21"/>
         <v>11420.08</v>
       </c>
-      <c r="S22" s="84">
+      <c r="S22" s="76">
         <v>0.25</v>
       </c>
-      <c r="T22" s="85">
+      <c r="T22" s="77">
         <v>0.0793</v>
       </c>
-      <c r="U22" s="85">
+      <c r="U22" s="77">
         <v>0.0477</v>
       </c>
-      <c r="V22" s="86">
+      <c r="V22" s="78">
         <v>0.0182</v>
       </c>
-      <c r="W22" s="81">
+      <c r="W22" s="75">
         <v>-0.0093</v>
       </c>
-      <c r="X22" s="79">
+      <c r="X22" s="73">
         <v>-0.0443</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="F23" s="12"/>
-      <c r="G23" s="20"/>
-      <c r="M23" s="15" t="s">
+      <c r="G23" s="19"/>
+      <c r="M23" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="N23" s="26">
+      <c r="N23" s="24">
         <v>0.0</v>
       </c>
-      <c r="O23" s="26">
+      <c r="O23" s="24">
         <v>6783.61</v>
       </c>
-      <c r="P23" s="26">
+      <c r="P23" s="24">
         <v>0.0</v>
       </c>
-      <c r="Q23" s="27">
+      <c r="Q23" s="25">
         <f t="shared" si="21"/>
         <v>6783.61</v>
       </c>
-      <c r="S23" s="76">
+      <c r="S23" s="70">
         <v>0.3</v>
       </c>
-      <c r="T23" s="77">
+      <c r="T23" s="71">
         <v>0.0745</v>
       </c>
-      <c r="U23" s="77">
+      <c r="U23" s="71">
         <v>0.042</v>
       </c>
-      <c r="V23" s="77">
+      <c r="V23" s="71">
         <v>0.0117</v>
       </c>
-      <c r="W23" s="81">
+      <c r="W23" s="75">
         <v>-0.0164</v>
       </c>
-      <c r="X23" s="79">
+      <c r="X23" s="73">
         <v>-0.0523</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="9" t="s">
         <v>92</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="3"/>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="G24" s="64">
+      <c r="G24" s="20">
         <v>0.015</v>
       </c>
       <c r="I24" s="11" t="s">
         <v>94</v>
       </c>
       <c r="J24" s="3"/>
-      <c r="M24" s="30" t="s">
+      <c r="M24" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="N24" s="50">
+      <c r="N24" s="35">
         <v>11474.05</v>
       </c>
-      <c r="O24" s="50">
+      <c r="O24" s="35">
         <v>537.87</v>
       </c>
-      <c r="P24" s="50">
+      <c r="P24" s="35">
         <v>0.0</v>
       </c>
-      <c r="Q24" s="33">
+      <c r="Q24" s="31">
         <f t="shared" si="21"/>
         <v>12011.92</v>
       </c>
-      <c r="S24" s="87">
+      <c r="S24" s="79">
         <v>0.35</v>
       </c>
-      <c r="T24" s="88">
+      <c r="T24" s="80">
         <v>0.0698</v>
       </c>
-      <c r="U24" s="88">
+      <c r="U24" s="80">
         <v>0.0364</v>
       </c>
-      <c r="V24" s="88">
+      <c r="V24" s="80">
         <v>0.0053</v>
       </c>
-      <c r="W24" s="89">
+      <c r="W24" s="81">
         <v>-0.0235</v>
       </c>
-      <c r="X24" s="90">
+      <c r="X24" s="82">
         <v>-0.0601</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="12"/>
       <c r="B25" s="13" t="s">
         <v>18</v>
@@ -2898,195 +2785,195 @@
       <c r="C25" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F25" s="30" t="s">
+      <c r="F25" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="G25" s="91">
+      <c r="G25" s="36">
         <v>0.01</v>
       </c>
-      <c r="I25" s="92" t="s">
+      <c r="I25" s="83" t="s">
         <v>97</v>
       </c>
       <c r="J25" s="8"/>
-      <c r="M25" s="36" t="s">
+      <c r="M25" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="N25" s="93">
+      <c r="N25" s="37">
         <f t="shared" ref="N25:Q25" si="24">SUM(N17:N24)</f>
         <v>181798.9</v>
       </c>
-      <c r="O25" s="40">
+      <c r="O25" s="37">
         <f t="shared" si="24"/>
         <v>121916.8</v>
       </c>
-      <c r="P25" s="40">
+      <c r="P25" s="37">
         <f t="shared" si="24"/>
         <v>8597.483025</v>
       </c>
-      <c r="Q25" s="55">
+      <c r="Q25" s="51">
         <f t="shared" si="24"/>
         <v>312313.183</v>
       </c>
-      <c r="S25" s="71" t="s">
+      <c r="S25" s="58" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="15" t="s">
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="18">
+      <c r="B26" s="17">
         <v>77452.0</v>
       </c>
-      <c r="C26" s="18">
+      <c r="C26" s="17">
         <v>80314.0</v>
       </c>
-      <c r="D26" s="94">
+      <c r="D26" s="15">
         <v>78124.0</v>
       </c>
-      <c r="F26" s="71" t="s">
+      <c r="F26" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="I26" s="15" t="s">
+      <c r="I26" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="J26" s="94">
+      <c r="J26" s="15">
         <v>5000.0</v>
       </c>
       <c r="M26" s="12"/>
-      <c r="N26" s="35"/>
-      <c r="O26" s="35"/>
-      <c r="P26" s="35"/>
-      <c r="Q26" s="20"/>
-      <c r="S26" s="71" t="s">
+      <c r="N26" s="32"/>
+      <c r="O26" s="32"/>
+      <c r="P26" s="32"/>
+      <c r="Q26" s="19"/>
+      <c r="S26" s="58" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="15" t="s">
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="26">
+      <c r="B27" s="24">
         <v>35453.0</v>
       </c>
-      <c r="C27" s="26">
+      <c r="C27" s="24">
         <v>37248.0</v>
       </c>
-      <c r="D27" s="95">
+      <c r="D27" s="25">
         <v>37197.0</v>
       </c>
-      <c r="F27" s="71" t="s">
+      <c r="F27" s="58" t="s">
         <v>103</v>
       </c>
-      <c r="I27" s="30" t="s">
+      <c r="I27" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="J27" s="96">
+      <c r="J27" s="31">
         <v>10000.0</v>
       </c>
-      <c r="K27" s="97"/>
-      <c r="M27" s="15" t="s">
+      <c r="K27" s="84"/>
+      <c r="M27" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="N27" s="18">
+      <c r="N27" s="17">
         <v>33805.07</v>
       </c>
-      <c r="O27" s="18">
+      <c r="O27" s="17">
         <v>24470.71</v>
       </c>
-      <c r="P27" s="23">
+      <c r="P27" s="21">
         <f>(-O27)+G8</f>
         <v>-18887.0418</v>
       </c>
-      <c r="Q27" s="16">
+      <c r="Q27" s="15">
         <f t="shared" ref="Q27:Q32" si="25">SUM(N27:P27)</f>
         <v>39388.7382</v>
       </c>
-      <c r="S27" s="71" t="s">
+      <c r="S27" s="58" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="15" t="s">
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="B28" s="26">
+      <c r="B28" s="24">
         <v>31059.0</v>
       </c>
-      <c r="C28" s="26">
+      <c r="C28" s="24">
         <v>32611.0</v>
       </c>
-      <c r="D28" s="95">
+      <c r="D28" s="25">
         <v>32467.0</v>
       </c>
-      <c r="F28" s="71" t="s">
+      <c r="F28" s="58" t="s">
         <v>108</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="I28" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="J28" s="16">
+      <c r="J28" s="15">
         <f>J26+J27</f>
         <v>15000</v>
       </c>
-      <c r="K28" s="98"/>
-      <c r="M28" s="15" t="s">
+      <c r="K28" s="85"/>
+      <c r="M28" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="N28" s="26">
+      <c r="N28" s="24">
         <v>0.0</v>
       </c>
-      <c r="O28" s="26">
+      <c r="O28" s="24">
         <v>80.0</v>
       </c>
-      <c r="P28" s="34">
+      <c r="P28" s="24">
         <f>-O28</f>
         <v>-80</v>
       </c>
-      <c r="Q28" s="27">
+      <c r="Q28" s="25">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="15" t="s">
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="B29" s="99">
+      <c r="B29" s="86">
         <v>21840.0</v>
       </c>
-      <c r="C29" s="26">
+      <c r="C29" s="24">
         <v>22931.0</v>
       </c>
-      <c r="D29" s="95">
+      <c r="D29" s="25">
         <v>22959.0</v>
       </c>
-      <c r="F29" s="71" t="s">
+      <c r="F29" s="58" t="s">
         <v>112</v>
       </c>
-      <c r="I29" s="30" t="s">
+      <c r="I29" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="J29" s="91">
+      <c r="J29" s="36">
         <v>0.25</v>
       </c>
-      <c r="M29" s="15" t="s">
+      <c r="M29" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="N29" s="26">
+      <c r="N29" s="24">
         <v>18233.48</v>
       </c>
-      <c r="O29" s="26">
+      <c r="O29" s="24">
         <v>5612.32</v>
       </c>
-      <c r="P29" s="34">
+      <c r="P29" s="24">
         <f>(-O29)+(D53-G8)</f>
         <v>1534.775298</v>
       </c>
-      <c r="Q29" s="27">
+      <c r="Q29" s="25">
         <f t="shared" si="25"/>
         <v>25380.5753</v>
       </c>
@@ -3099,47 +2986,47 @@
       <c r="W29" s="2"/>
       <c r="X29" s="3"/>
     </row>
-    <row r="30">
-      <c r="A30" s="15" t="s">
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="B30" s="100">
+      <c r="B30" s="87">
         <v>0.6685</v>
       </c>
-      <c r="C30" s="100">
+      <c r="C30" s="87">
         <v>0.7012</v>
       </c>
-      <c r="D30" s="101">
+      <c r="D30" s="88">
         <v>0.7174</v>
       </c>
-      <c r="F30" s="71" t="s">
+      <c r="F30" s="58" t="s">
         <v>117</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="I30" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="J30" s="16">
+      <c r="J30" s="15">
         <f>J28*J29</f>
         <v>3750</v>
       </c>
-      <c r="M30" s="15" t="s">
+      <c r="M30" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="N30" s="26">
+      <c r="N30" s="24">
         <v>-3117.82</v>
       </c>
-      <c r="O30" s="26">
+      <c r="O30" s="24">
         <v>-2078.08</v>
       </c>
-      <c r="P30" s="34">
+      <c r="P30" s="24">
         <f>ABS(O30)</f>
         <v>2078.08</v>
       </c>
-      <c r="Q30" s="27">
+      <c r="Q30" s="25">
         <f t="shared" si="25"/>
         <v>-3117.82</v>
       </c>
-      <c r="S30" s="68"/>
+      <c r="S30" s="63"/>
       <c r="T30" s="13" t="s">
         <v>120</v>
       </c>
@@ -3148,386 +3035,386 @@
       <c r="W30" s="7"/>
       <c r="X30" s="8"/>
     </row>
-    <row r="31">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="12"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="20"/>
-      <c r="F31" s="71" t="s">
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="19"/>
+      <c r="F31" s="58" t="s">
         <v>121</v>
       </c>
-      <c r="I31" s="15"/>
-      <c r="J31" s="20"/>
-      <c r="M31" s="15" t="s">
+      <c r="I31" s="12"/>
+      <c r="J31" s="19"/>
+      <c r="M31" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="N31" s="26">
+      <c r="N31" s="24">
         <v>22054.26</v>
       </c>
-      <c r="O31" s="26">
+      <c r="O31" s="24">
         <v>414.59</v>
       </c>
-      <c r="P31" s="34">
+      <c r="P31" s="24">
         <f>-O31</f>
         <v>-414.59</v>
       </c>
-      <c r="Q31" s="27">
+      <c r="Q31" s="25">
         <f t="shared" si="25"/>
         <v>22054.26</v>
       </c>
-      <c r="S31" s="102" t="s">
+      <c r="S31" s="89" t="s">
         <v>123</v>
       </c>
-      <c r="T31" s="103">
+      <c r="T31" s="90">
         <v>0.0575</v>
       </c>
-      <c r="U31" s="103">
+      <c r="U31" s="90">
         <v>0.0625</v>
       </c>
-      <c r="V31" s="104">
+      <c r="V31" s="91">
         <v>0.0675</v>
       </c>
-      <c r="W31" s="103">
+      <c r="W31" s="90">
         <v>0.0725</v>
       </c>
-      <c r="X31" s="105">
+      <c r="X31" s="92">
         <v>0.0775</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="15" t="s">
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="18">
+      <c r="B32" s="17">
         <v>25271.0</v>
       </c>
-      <c r="C32" s="18">
+      <c r="C32" s="17">
         <v>25713.0</v>
       </c>
-      <c r="D32" s="94">
+      <c r="D32" s="15">
         <v>25090.0</v>
       </c>
-      <c r="F32" s="71" t="s">
+      <c r="F32" s="58" t="s">
         <v>125</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="I32" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="J32" s="16">
+      <c r="J32" s="15">
         <f>J28-J30</f>
         <v>11250</v>
       </c>
-      <c r="M32" s="30" t="s">
+      <c r="M32" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="N32" s="50">
+      <c r="N32" s="35">
         <v>213374.76</v>
       </c>
-      <c r="O32" s="50">
+      <c r="O32" s="35">
         <v>64119.36</v>
       </c>
-      <c r="P32" s="38">
+      <c r="P32" s="35">
         <f>(-O32)-J9+J44</f>
         <v>15302.72315</v>
       </c>
-      <c r="Q32" s="33">
+      <c r="Q32" s="31">
         <f t="shared" si="25"/>
         <v>292796.8432</v>
       </c>
-      <c r="S32" s="106">
+      <c r="S32" s="93">
         <v>0.0</v>
       </c>
-      <c r="T32" s="77">
+      <c r="T32" s="71">
         <v>0.0041</v>
       </c>
-      <c r="U32" s="77">
+      <c r="U32" s="71">
         <v>0.0034</v>
       </c>
-      <c r="V32" s="78">
+      <c r="V32" s="72">
         <v>0.0027</v>
       </c>
-      <c r="W32" s="77">
+      <c r="W32" s="71">
         <v>0.002</v>
       </c>
-      <c r="X32" s="107">
+      <c r="X32" s="94">
         <v>0.0013</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="15" t="s">
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B33" s="26">
+      <c r="B33" s="24">
         <v>10677.0</v>
       </c>
-      <c r="C33" s="26">
+      <c r="C33" s="24">
         <v>10813.0</v>
       </c>
-      <c r="D33" s="95">
+      <c r="D33" s="25">
         <v>11066.0</v>
       </c>
-      <c r="F33" s="71" t="s">
+      <c r="F33" s="58" t="s">
         <v>129</v>
       </c>
-      <c r="I33" s="108"/>
-      <c r="J33" s="109"/>
-      <c r="K33" s="71"/>
-      <c r="M33" s="15" t="s">
+      <c r="I33" s="95"/>
+      <c r="J33" s="96"/>
+      <c r="K33" s="58"/>
+      <c r="M33" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="N33" s="21">
+      <c r="N33" s="17">
         <f t="shared" ref="N33:O33" si="26">B22</f>
         <v>284350.55</v>
       </c>
-      <c r="O33" s="21">
+      <c r="O33" s="17">
         <f t="shared" si="26"/>
         <v>92618.9</v>
       </c>
-      <c r="P33" s="23">
+      <c r="P33" s="21">
         <f t="shared" ref="P33:Q33" si="27">SUM(P27:P32)</f>
         <v>-466.05335</v>
       </c>
-      <c r="Q33" s="16">
+      <c r="Q33" s="15">
         <f t="shared" si="27"/>
         <v>376502.5967</v>
       </c>
-      <c r="S33" s="106">
+      <c r="S33" s="93">
         <v>325.0</v>
       </c>
-      <c r="T33" s="77">
+      <c r="T33" s="71">
         <v>0.011</v>
       </c>
-      <c r="U33" s="77">
+      <c r="U33" s="71">
         <v>0.0103</v>
       </c>
-      <c r="V33" s="78">
+      <c r="V33" s="72">
         <v>0.0096</v>
       </c>
-      <c r="W33" s="77">
+      <c r="W33" s="71">
         <v>0.0089</v>
       </c>
-      <c r="X33" s="107">
+      <c r="X33" s="94">
         <v>0.0082</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="15" t="s">
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="B34" s="26">
+      <c r="B34" s="24">
         <v>8903.0</v>
       </c>
-      <c r="C34" s="26">
+      <c r="C34" s="24">
         <v>8842.0</v>
       </c>
-      <c r="D34" s="95">
+      <c r="D34" s="25">
         <v>8841.0</v>
       </c>
-      <c r="F34" s="71" t="s">
+      <c r="F34" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="I34" s="92" t="s">
+      <c r="I34" s="83" t="s">
         <v>133</v>
       </c>
       <c r="J34" s="8"/>
-      <c r="M34" s="30" t="s">
+      <c r="M34" s="28" t="s">
         <v>134</v>
       </c>
-      <c r="N34" s="50">
+      <c r="N34" s="35">
         <v>36316.77</v>
       </c>
-      <c r="O34" s="50">
+      <c r="O34" s="35">
         <v>4504.58</v>
       </c>
-      <c r="P34" s="50">
+      <c r="P34" s="35">
         <v>0.0</v>
       </c>
-      <c r="Q34" s="33">
+      <c r="Q34" s="31">
         <f>SUM(N34:P34)</f>
         <v>40821.35</v>
       </c>
-      <c r="S34" s="110">
+      <c r="S34" s="97">
         <v>650.0</v>
       </c>
-      <c r="T34" s="85">
+      <c r="T34" s="77">
         <v>0.0178</v>
       </c>
-      <c r="U34" s="85">
+      <c r="U34" s="77">
         <v>0.0171</v>
       </c>
-      <c r="V34" s="86">
+      <c r="V34" s="78">
         <v>0.0164</v>
       </c>
-      <c r="W34" s="77">
+      <c r="W34" s="71">
         <v>0.0157</v>
       </c>
-      <c r="X34" s="107">
+      <c r="X34" s="94">
         <v>0.0151</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="15" t="s">
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="B35" s="26">
+      <c r="B35" s="24">
         <v>4255.0</v>
       </c>
-      <c r="C35" s="26">
+      <c r="C35" s="24">
         <v>4138.0</v>
       </c>
-      <c r="D35" s="95">
+      <c r="D35" s="25">
         <v>3960.0</v>
       </c>
-      <c r="F35" s="71" t="s">
+      <c r="F35" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="I35" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J35" s="16">
+      <c r="J35" s="15">
         <f>D43</f>
         <v>19585.79</v>
       </c>
-      <c r="M35" s="111" t="s">
+      <c r="M35" s="98" t="s">
         <v>82</v>
       </c>
-      <c r="N35" s="112">
+      <c r="N35" s="99">
         <f t="shared" ref="N35:Q35" si="28">N33+N34</f>
         <v>320667.32</v>
       </c>
-      <c r="O35" s="112">
+      <c r="O35" s="99">
         <f t="shared" si="28"/>
         <v>97123.48</v>
       </c>
-      <c r="P35" s="113">
+      <c r="P35" s="100">
         <f t="shared" si="28"/>
         <v>-466.05335</v>
       </c>
-      <c r="Q35" s="114">
+      <c r="Q35" s="101">
         <f t="shared" si="28"/>
         <v>417323.9467</v>
       </c>
-      <c r="S35" s="106">
+      <c r="S35" s="93">
         <v>975.0</v>
       </c>
-      <c r="T35" s="77">
+      <c r="T35" s="71">
         <v>0.0247</v>
       </c>
-      <c r="U35" s="77">
+      <c r="U35" s="71">
         <v>0.024</v>
       </c>
-      <c r="V35" s="77">
+      <c r="V35" s="71">
         <v>0.0233</v>
       </c>
-      <c r="W35" s="77">
+      <c r="W35" s="71">
         <v>0.0226</v>
       </c>
-      <c r="X35" s="107">
+      <c r="X35" s="94">
         <v>0.0219</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="30" t="s">
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B36" s="115">
+      <c r="B36" s="102">
         <v>0.1886</v>
       </c>
-      <c r="C36" s="115">
+      <c r="C36" s="102">
         <v>0.18</v>
       </c>
-      <c r="D36" s="116">
+      <c r="D36" s="103">
         <v>0.1769</v>
       </c>
-      <c r="F36" s="71" t="s">
+      <c r="F36" s="58" t="s">
         <v>138</v>
       </c>
       <c r="I36" s="12"/>
-      <c r="J36" s="20"/>
-      <c r="M36" s="117"/>
-      <c r="N36" s="118"/>
-      <c r="O36" s="118"/>
-      <c r="P36" s="118"/>
-      <c r="Q36" s="119"/>
-      <c r="S36" s="120">
+      <c r="J36" s="19"/>
+      <c r="M36" s="104"/>
+      <c r="N36" s="105"/>
+      <c r="O36" s="105"/>
+      <c r="P36" s="105"/>
+      <c r="Q36" s="106"/>
+      <c r="S36" s="107">
         <v>1300.0</v>
       </c>
-      <c r="T36" s="88">
+      <c r="T36" s="80">
         <v>0.0315</v>
       </c>
-      <c r="U36" s="88">
+      <c r="U36" s="80">
         <v>0.0308</v>
       </c>
-      <c r="V36" s="88">
+      <c r="V36" s="80">
         <v>0.0301</v>
       </c>
-      <c r="W36" s="88">
+      <c r="W36" s="80">
         <v>0.0295</v>
       </c>
-      <c r="X36" s="121">
+      <c r="X36" s="108">
         <v>0.0288</v>
       </c>
     </row>
-    <row r="37">
-      <c r="F37" s="71" t="s">
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="F37" s="58" t="s">
         <v>139</v>
       </c>
-      <c r="I37" s="15" t="s">
+      <c r="I37" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="J37" s="27">
+      <c r="J37" s="25">
         <f>C22</f>
         <v>92618.9</v>
       </c>
-      <c r="M37" s="111" t="s">
+      <c r="M37" s="98" t="s">
         <v>141</v>
       </c>
-      <c r="N37" s="122">
+      <c r="N37" s="99">
         <f t="shared" ref="N37:P37" si="29">N25+N35</f>
         <v>502466.22</v>
       </c>
-      <c r="O37" s="112">
+      <c r="O37" s="99">
         <f t="shared" si="29"/>
         <v>219040.28</v>
       </c>
-      <c r="P37" s="112">
+      <c r="P37" s="99">
         <f t="shared" si="29"/>
         <v>8131.429675</v>
       </c>
-      <c r="Q37" s="123">
+      <c r="Q37" s="101">
         <f>SUM(N37:P37)</f>
         <v>729637.9297</v>
       </c>
-      <c r="S37" s="71" t="s">
+      <c r="S37" s="58" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="15.75" customHeight="1">
       <c r="B38" s="10" t="s">
         <v>142</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="3"/>
-      <c r="I38" s="15" t="s">
+      <c r="I38" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="J38" s="95">
+      <c r="J38" s="25">
         <v>4567.24</v>
       </c>
       <c r="M38" s="12"/>
-      <c r="N38" s="35"/>
-      <c r="O38" s="35"/>
-      <c r="P38" s="35"/>
-      <c r="Q38" s="20"/>
-      <c r="S38" s="71" t="s">
+      <c r="N38" s="32"/>
+      <c r="O38" s="32"/>
+      <c r="P38" s="32"/>
+      <c r="Q38" s="19"/>
+      <c r="S38" s="58" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="15" t="s">
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="B39" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="D39" s="16">
+      <c r="D39" s="15">
         <f>C7</f>
         <v>0.7</v>
       </c>
@@ -3535,71 +3422,71 @@
         <v>146</v>
       </c>
       <c r="G39" s="3"/>
-      <c r="I39" s="30" t="s">
+      <c r="I39" s="28" t="s">
         <v>147</v>
       </c>
-      <c r="J39" s="33">
+      <c r="J39" s="31">
         <f>J32</f>
         <v>11250</v>
       </c>
-      <c r="M39" s="65" t="s">
+      <c r="M39" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="N39" s="66">
+      <c r="N39" s="61">
         <f t="shared" ref="N39:Q39" si="30">N15-N37</f>
         <v>0</v>
       </c>
-      <c r="O39" s="66">
+      <c r="O39" s="61">
         <f t="shared" si="30"/>
         <v>0</v>
       </c>
-      <c r="P39" s="124">
+      <c r="P39" s="109">
         <f t="shared" si="30"/>
         <v>0</v>
       </c>
-      <c r="Q39" s="125">
+      <c r="Q39" s="110">
         <f t="shared" si="30"/>
         <v>0</v>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="30" t="s">
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="B40" s="28" t="s">
         <v>148</v>
       </c>
       <c r="C40" s="7"/>
-      <c r="D40" s="91">
+      <c r="D40" s="36">
         <v>0.25</v>
       </c>
-      <c r="F40" s="15" t="s">
+      <c r="F40" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="G40" s="94">
+      <c r="G40" s="15">
         <v>650.0</v>
       </c>
-      <c r="I40" s="15" t="s">
+      <c r="I40" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="J40" s="126">
+      <c r="J40" s="111">
         <f>J37-J38+J39</f>
         <v>99301.66</v>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" s="36" t="s">
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="B41" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="D41" s="55">
+      <c r="D41" s="51">
         <f>D39*(1+D40)</f>
         <v>0.875</v>
       </c>
-      <c r="F41" s="15" t="s">
+      <c r="F41" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="G41" s="64">
+      <c r="G41" s="20">
         <v>0.25</v>
       </c>
       <c r="I41" s="12"/>
-      <c r="J41" s="20"/>
+      <c r="J41" s="19"/>
       <c r="M41" s="11" t="s">
         <v>153</v>
       </c>
@@ -3607,25 +3494,25 @@
       <c r="O41" s="2"/>
       <c r="P41" s="3"/>
     </row>
-    <row r="42">
-      <c r="B42" s="30" t="s">
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="B42" s="28" t="s">
         <v>154</v>
       </c>
       <c r="C42" s="7"/>
-      <c r="D42" s="33">
+      <c r="D42" s="31">
         <f>C8</f>
         <v>22383.76</v>
       </c>
-      <c r="F42" s="15" t="s">
+      <c r="F42" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="G42" s="64">
+      <c r="G42" s="20">
         <v>0.75</v>
       </c>
-      <c r="I42" s="15" t="s">
+      <c r="I42" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="J42" s="127">
+      <c r="J42" s="111">
         <f>J35-J40</f>
         <v>-79715.87</v>
       </c>
@@ -3636,455 +3523,1403 @@
       <c r="O42" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="P42" s="17" t="s">
+      <c r="P42" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="128" t="s">
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="B43" s="112" t="s">
         <v>157</v>
       </c>
       <c r="C43" s="7"/>
-      <c r="D43" s="129">
+      <c r="D43" s="113">
         <f>D41*D42</f>
         <v>19585.79</v>
       </c>
-      <c r="F43" s="30" t="s">
+      <c r="F43" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="G43" s="91">
+      <c r="G43" s="36">
         <v>1.0</v>
       </c>
-      <c r="I43" s="36" t="s">
+      <c r="I43" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="J43" s="55">
+      <c r="J43" s="51">
         <f>MAX(0, J35-J40)</f>
         <v>0</v>
       </c>
-      <c r="M43" s="15" t="s">
+      <c r="M43" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="N43" s="21">
+      <c r="N43" s="17">
         <f t="shared" ref="N43:P43" si="31">B29</f>
         <v>21840</v>
       </c>
-      <c r="O43" s="21">
+      <c r="O43" s="17">
         <f t="shared" si="31"/>
         <v>22931</v>
       </c>
-      <c r="P43" s="16">
+      <c r="P43" s="15">
         <f t="shared" si="31"/>
         <v>22959</v>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="71" t="s">
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="B44" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="F44" s="71" t="s">
+      <c r="F44" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="I44" s="130" t="s">
+      <c r="I44" s="114" t="s">
         <v>161</v>
       </c>
-      <c r="J44" s="131">
+      <c r="J44" s="115">
         <f>MAX(0, J40-J35)</f>
         <v>79715.87</v>
       </c>
-      <c r="M44" s="30" t="s">
+      <c r="M44" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="N44" s="38">
+      <c r="N44" s="35">
         <f t="shared" ref="N44:P44" si="32">B35</f>
         <v>4255</v>
       </c>
-      <c r="O44" s="38">
+      <c r="O44" s="35">
         <f t="shared" si="32"/>
         <v>4138</v>
       </c>
-      <c r="P44" s="33">
+      <c r="P44" s="31">
         <f t="shared" si="32"/>
         <v>3960</v>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="132" t="s">
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="B45" s="116" t="s">
         <v>163</v>
       </c>
-      <c r="F45" s="71" t="s">
+      <c r="F45" s="58" t="s">
         <v>164</v>
       </c>
-      <c r="I45" s="71" t="s">
+      <c r="I45" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="M45" s="15" t="s">
+      <c r="M45" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="N45" s="21">
+      <c r="N45" s="17">
         <f t="shared" ref="N45:P45" si="33">N43+N44</f>
         <v>26095</v>
       </c>
-      <c r="O45" s="21">
+      <c r="O45" s="17">
         <f t="shared" si="33"/>
         <v>27069</v>
       </c>
-      <c r="P45" s="16">
+      <c r="P45" s="15">
         <f t="shared" si="33"/>
         <v>26919</v>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="71" t="s">
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="B46" s="58" t="s">
         <v>166</v>
       </c>
-      <c r="F46" s="71" t="s">
+      <c r="F46" s="58" t="s">
         <v>167</v>
       </c>
-      <c r="I46" s="71" t="s">
+      <c r="I46" s="58" t="s">
         <v>168</v>
       </c>
       <c r="M46" s="12"/>
-      <c r="N46" s="35"/>
-      <c r="O46" s="35"/>
-      <c r="P46" s="20"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="71" t="s">
+      <c r="N46" s="32"/>
+      <c r="O46" s="32"/>
+      <c r="P46" s="19"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="B47" s="58" t="s">
         <v>169</v>
       </c>
-      <c r="F47" s="71" t="s">
+      <c r="F47" s="58" t="s">
         <v>170</v>
       </c>
-      <c r="I47" s="71" t="s">
+      <c r="I47" s="58" t="s">
         <v>171</v>
       </c>
-      <c r="M47" s="133" t="s">
+      <c r="M47" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="N47" s="35"/>
-      <c r="O47" s="35"/>
-      <c r="P47" s="20"/>
-    </row>
-    <row r="48">
-      <c r="B48" s="71"/>
-      <c r="C48" s="71"/>
-      <c r="D48" s="71"/>
-      <c r="F48" s="71" t="s">
+      <c r="N47" s="32"/>
+      <c r="O47" s="32"/>
+      <c r="P47" s="19"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="B48" s="58"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="F48" s="58" t="s">
         <v>173</v>
       </c>
-      <c r="I48" s="71" t="s">
+      <c r="I48" s="58" t="s">
         <v>174</v>
       </c>
-      <c r="M48" s="15" t="s">
+      <c r="M48" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="N48" s="21">
+      <c r="N48" s="17">
         <f>G40*G41</f>
         <v>162.5</v>
       </c>
-      <c r="O48" s="21">
+      <c r="O48" s="17">
         <f>G40*G42</f>
         <v>487.5</v>
       </c>
-      <c r="P48" s="16">
+      <c r="P48" s="15">
         <f>G40*G43</f>
         <v>650</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="15.75" customHeight="1">
       <c r="B49" s="10" t="s">
         <v>176</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="3"/>
-      <c r="F49" s="71" t="s">
+      <c r="F49" s="58" t="s">
         <v>177</v>
       </c>
-      <c r="I49" s="71"/>
-      <c r="M49" s="15" t="s">
+      <c r="I49" s="58"/>
+      <c r="M49" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="N49" s="34">
+      <c r="N49" s="24">
         <f t="shared" ref="N49:P49" si="34">-($J$13*$G$18)</f>
         <v>-330.5102063</v>
       </c>
-      <c r="O49" s="34">
+      <c r="O49" s="24">
         <f t="shared" si="34"/>
         <v>-330.5102063</v>
       </c>
-      <c r="P49" s="27">
+      <c r="P49" s="25">
         <f t="shared" si="34"/>
         <v>-330.5102063</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="15.75" customHeight="1">
       <c r="B50" s="12"/>
       <c r="C50" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="D50" s="17" t="s">
+      <c r="D50" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F50" s="71" t="s">
+      <c r="F50" s="58" t="s">
         <v>181</v>
       </c>
-      <c r="I50" s="71"/>
-      <c r="M50" s="15" t="s">
+      <c r="I50" s="58"/>
+      <c r="M50" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="N50" s="34">
+      <c r="N50" s="24">
         <f t="shared" ref="N50:P50" si="35">-($J$10/5)</f>
         <v>-9.792895</v>
       </c>
-      <c r="O50" s="34">
+      <c r="O50" s="24">
         <f t="shared" si="35"/>
         <v>-9.792895</v>
       </c>
-      <c r="P50" s="27">
+      <c r="P50" s="25">
         <f t="shared" si="35"/>
         <v>-9.792895</v>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="15" t="s">
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="B51" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="C51" s="134">
+      <c r="C51" s="118">
         <v>0.1</v>
       </c>
-      <c r="D51" s="16">
+      <c r="D51" s="15">
         <f t="shared" ref="D51:D53" si="37">$D$43*C51</f>
         <v>1958.579</v>
       </c>
-      <c r="F51" s="71" t="s">
+      <c r="F51" s="58" t="s">
         <v>184</v>
       </c>
-      <c r="I51" s="71"/>
-      <c r="M51" s="30" t="s">
+      <c r="I51" s="58"/>
+      <c r="M51" s="28" t="s">
         <v>185</v>
       </c>
-      <c r="N51" s="38">
+      <c r="N51" s="35">
         <f t="shared" ref="N51:P51" si="36">-($J$15*$G$19)</f>
         <v>-115.0665163</v>
       </c>
-      <c r="O51" s="38">
+      <c r="O51" s="35">
         <f t="shared" si="36"/>
         <v>-115.0665163</v>
       </c>
-      <c r="P51" s="33">
+      <c r="P51" s="31">
         <f t="shared" si="36"/>
         <v>-115.0665163</v>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="15" t="s">
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="B52" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="C52" s="134">
+      <c r="C52" s="118">
         <v>0.25</v>
       </c>
-      <c r="D52" s="16">
+      <c r="D52" s="15">
         <f t="shared" si="37"/>
         <v>4896.4475</v>
       </c>
-      <c r="I52" s="71"/>
-      <c r="M52" s="15" t="s">
+      <c r="I52" s="58"/>
+      <c r="M52" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="N52" s="23">
+      <c r="N52" s="21">
         <f t="shared" ref="N52:P52" si="38">SUM(N48:N51)</f>
         <v>-292.8696175</v>
       </c>
-      <c r="O52" s="23">
+      <c r="O52" s="21">
         <f t="shared" si="38"/>
         <v>32.1303825</v>
       </c>
-      <c r="P52" s="127">
+      <c r="P52" s="111">
         <f t="shared" si="38"/>
         <v>194.6303825</v>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="30" t="s">
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="B53" s="28" t="s">
         <v>188</v>
       </c>
-      <c r="C53" s="135">
+      <c r="C53" s="119">
         <v>0.65</v>
       </c>
-      <c r="D53" s="136">
+      <c r="D53" s="120">
         <f t="shared" si="37"/>
         <v>12730.7635</v>
       </c>
-      <c r="I53" s="71"/>
-      <c r="M53" s="30" t="s">
+      <c r="I53" s="58"/>
+      <c r="M53" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="N53" s="38">
+      <c r="N53" s="35">
         <f t="shared" ref="N53:P53" si="39">N52*$G$20</f>
         <v>-73.21740438</v>
       </c>
-      <c r="O53" s="38">
+      <c r="O53" s="35">
         <f t="shared" si="39"/>
         <v>8.032595625</v>
       </c>
-      <c r="P53" s="33">
+      <c r="P53" s="31">
         <f t="shared" si="39"/>
         <v>48.65759563</v>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="128" t="s">
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="B54" s="112" t="s">
         <v>190</v>
       </c>
-      <c r="C54" s="137">
+      <c r="C54" s="121">
         <f t="shared" ref="C54:D54" si="40">SUM(C51:C53)</f>
         <v>1</v>
       </c>
-      <c r="D54" s="129">
+      <c r="D54" s="113">
         <f t="shared" si="40"/>
         <v>19585.79</v>
       </c>
-      <c r="M54" s="15" t="s">
+      <c r="M54" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="N54" s="23">
+      <c r="N54" s="21">
         <f t="shared" ref="N54:P54" si="41">N52-N53</f>
         <v>-219.6522131</v>
       </c>
-      <c r="O54" s="23">
+      <c r="O54" s="21">
         <f t="shared" si="41"/>
         <v>24.09778688</v>
       </c>
-      <c r="P54" s="127">
+      <c r="P54" s="111">
         <f t="shared" si="41"/>
         <v>145.9727869</v>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" s="71" t="s">
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="B55" s="58" t="s">
         <v>76</v>
       </c>
       <c r="M55" s="12"/>
-      <c r="N55" s="35"/>
-      <c r="O55" s="35"/>
-      <c r="P55" s="20"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="71" t="s">
+      <c r="N55" s="32"/>
+      <c r="O55" s="32"/>
+      <c r="P55" s="19"/>
+    </row>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="B56" s="58" t="s">
         <v>192</v>
       </c>
-      <c r="M56" s="128" t="s">
+      <c r="M56" s="112" t="s">
         <v>193</v>
       </c>
-      <c r="N56" s="138">
+      <c r="N56" s="122">
         <f t="shared" ref="N56:P56" si="42">N45+N54</f>
         <v>25875.34779</v>
       </c>
-      <c r="O56" s="138">
+      <c r="O56" s="122">
         <f t="shared" si="42"/>
         <v>27093.09779</v>
       </c>
-      <c r="P56" s="129">
+      <c r="P56" s="113">
         <f t="shared" si="42"/>
         <v>27064.97279</v>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="71" t="s">
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="B57" s="58" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="71" t="s">
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="B58" s="58" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="71" t="s">
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="B59" s="58" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="71" t="s">
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="B60" s="58" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="61">
-      <c r="B61" s="71" t="s">
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="B61" s="58" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" s="71" t="s">
+    <row r="62" ht="15.75" customHeight="1">
+      <c r="B62" s="58" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" s="71" t="s">
+    <row r="63" ht="15.75" customHeight="1">
+      <c r="B63" s="58" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="64">
-      <c r="B64" s="71" t="s">
+    <row r="64" ht="15.75" customHeight="1">
+      <c r="B64" s="58" t="s">
         <v>201</v>
       </c>
     </row>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
+    <row r="101" ht="15.75" customHeight="1"/>
+    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1"/>
+    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1"/>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="110" ht="15.75" customHeight="1"/>
+    <row r="111" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1"/>
+    <row r="113" ht="15.75" customHeight="1"/>
+    <row r="114" ht="15.75" customHeight="1"/>
+    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="117" ht="15.75" customHeight="1"/>
+    <row r="118" ht="15.75" customHeight="1"/>
+    <row r="119" ht="15.75" customHeight="1"/>
+    <row r="120" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1"/>
+    <row r="122" ht="15.75" customHeight="1"/>
+    <row r="123" ht="15.75" customHeight="1"/>
+    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="125" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1"/>
+    <row r="127" ht="15.75" customHeight="1"/>
+    <row r="128" ht="15.75" customHeight="1"/>
+    <row r="129" ht="15.75" customHeight="1"/>
+    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="131" ht="15.75" customHeight="1"/>
+    <row r="132" ht="15.75" customHeight="1"/>
+    <row r="133" ht="15.75" customHeight="1"/>
+    <row r="134" ht="15.75" customHeight="1"/>
+    <row r="135" ht="15.75" customHeight="1"/>
+    <row r="136" ht="15.75" customHeight="1"/>
+    <row r="137" ht="15.75" customHeight="1"/>
+    <row r="138" ht="15.75" customHeight="1"/>
+    <row r="139" ht="15.75" customHeight="1"/>
+    <row r="140" ht="15.75" customHeight="1"/>
+    <row r="141" ht="15.75" customHeight="1"/>
+    <row r="142" ht="15.75" customHeight="1"/>
+    <row r="143" ht="15.75" customHeight="1"/>
+    <row r="144" ht="15.75" customHeight="1"/>
+    <row r="145" ht="15.75" customHeight="1"/>
+    <row r="146" ht="15.75" customHeight="1"/>
+    <row r="147" ht="15.75" customHeight="1"/>
+    <row r="148" ht="15.75" customHeight="1"/>
+    <row r="149" ht="15.75" customHeight="1"/>
+    <row r="150" ht="15.75" customHeight="1"/>
+    <row r="151" ht="15.75" customHeight="1"/>
+    <row r="152" ht="15.75" customHeight="1"/>
+    <row r="153" ht="15.75" customHeight="1"/>
+    <row r="154" ht="15.75" customHeight="1"/>
+    <row r="155" ht="15.75" customHeight="1"/>
+    <row r="156" ht="15.75" customHeight="1"/>
+    <row r="157" ht="15.75" customHeight="1"/>
+    <row r="158" ht="15.75" customHeight="1"/>
+    <row r="159" ht="15.75" customHeight="1"/>
+    <row r="160" ht="15.75" customHeight="1"/>
+    <row r="161" ht="15.75" customHeight="1"/>
+    <row r="162" ht="15.75" customHeight="1"/>
+    <row r="163" ht="15.75" customHeight="1"/>
+    <row r="164" ht="15.75" customHeight="1"/>
+    <row r="165" ht="15.75" customHeight="1"/>
+    <row r="166" ht="15.75" customHeight="1"/>
+    <row r="167" ht="15.75" customHeight="1"/>
+    <row r="168" ht="15.75" customHeight="1"/>
+    <row r="169" ht="15.75" customHeight="1"/>
+    <row r="170" ht="15.75" customHeight="1"/>
+    <row r="171" ht="15.75" customHeight="1"/>
+    <row r="172" ht="15.75" customHeight="1"/>
+    <row r="173" ht="15.75" customHeight="1"/>
+    <row r="174" ht="15.75" customHeight="1"/>
+    <row r="175" ht="15.75" customHeight="1"/>
+    <row r="176" ht="15.75" customHeight="1"/>
+    <row r="177" ht="15.75" customHeight="1"/>
+    <row r="178" ht="15.75" customHeight="1"/>
+    <row r="179" ht="15.75" customHeight="1"/>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="91">
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
+    <mergeCell ref="M41:P41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="F44:G44"/>
+    <mergeCell ref="B45:D45"/>
     <mergeCell ref="F45:G45"/>
     <mergeCell ref="I45:J45"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="F50:G50"/>
     <mergeCell ref="I50:J50"/>
+    <mergeCell ref="F51:G51"/>
     <mergeCell ref="I51:J51"/>
     <mergeCell ref="I52:J52"/>
     <mergeCell ref="I53:J53"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B58:D58"/>
     <mergeCell ref="B59:D59"/>
     <mergeCell ref="B60:D60"/>
     <mergeCell ref="B61:D61"/>
     <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A2:W2"/>
+    <mergeCell ref="A3:W3"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="S5:W5"/>
     <mergeCell ref="S6:T6"/>
     <mergeCell ref="S7:T7"/>
     <mergeCell ref="S8:T8"/>
     <mergeCell ref="S9:T9"/>
     <mergeCell ref="S10:T10"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="S11:T11"/>
-    <mergeCell ref="S5:W5"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="S13:T13"/>
+    <mergeCell ref="F14:G14"/>
     <mergeCell ref="S14:T14"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="S17:X17"/>
-    <mergeCell ref="T18:X18"/>
-    <mergeCell ref="S25:X25"/>
-    <mergeCell ref="S27:X27"/>
-    <mergeCell ref="S26:X26"/>
-    <mergeCell ref="T30:X30"/>
-    <mergeCell ref="S29:X29"/>
-    <mergeCell ref="S37:X37"/>
-    <mergeCell ref="S38:X38"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="I19:K19"/>
@@ -4101,28 +4936,16 @@
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="M41:P41"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A1:W1"/>
-    <mergeCell ref="A2:W2"/>
-    <mergeCell ref="A3:W3"/>
+    <mergeCell ref="T30:X30"/>
+    <mergeCell ref="S37:X37"/>
+    <mergeCell ref="S38:X38"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="S17:X17"/>
+    <mergeCell ref="T18:X18"/>
+    <mergeCell ref="S25:X25"/>
+    <mergeCell ref="S26:X26"/>
+    <mergeCell ref="S27:X27"/>
+    <mergeCell ref="S29:X29"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>